<commit_message>
Update Excel column width for improved readability in IPO tracker
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -461,7 +461,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>last_updated_utc</t>
+          <t>last_updated_ist</t>
         </is>
       </c>
     </row>
@@ -617,11 +617,7 @@
           <t>https://www.moneycontrol.com/ipo/renewables/junipergreenenergy/JGE</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2026-08-07 11:09:00</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -687,11 +683,7 @@
           <t>https://www.moneycontrol.com/ipo/electric-equipment-switchgears/mvelectrosystems/MEL04</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2026-08-07 11:09:00</t>
-        </is>
-      </c>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -755,7 +747,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -821,7 +813,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -887,7 +879,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -949,7 +941,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1003,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1065,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1127,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1189,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-08-07 11:17:22</t>
+          <t>2026-08-07 16:49:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update IPO tracker data
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -747,7 +747,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-08-07 16:49:33</t>
+          <t>2026-08-07 21:39:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: set ipo allotment for LEAP India Ltd
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -570,15 +570,11 @@
           <t>Juniper Green Energy</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Listed</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Aug 06, 2026</t>
@@ -629,7 +625,6 @@
           <t>https://www.moneycontrol.com/ipo/renewables/junipergreenenergy/JGE</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -637,15 +632,11 @@
           <t>MV Electrosystems</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Listed</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Aug 06, 2026</t>
@@ -696,7 +687,6 @@
           <t>https://www.moneycontrol.com/ipo/electric-equipment-switchgears/mvelectrosystems/MEL04</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -704,14 +694,11 @@
           <t>Anawil Wire &amp; Engineering</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Listed</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Aug 06, 2025</t>
@@ -737,15 +724,11 @@
           <t>108000</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>139</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/infrastructure/anawilwireengineering/AWEL</t>
@@ -763,14 +746,11 @@
           <t>Ardee Industries</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Listed</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Aug 10, 2026</t>
@@ -796,15 +776,11 @@
           <t>14893</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>134</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/metals-non-ferrous/ardeeindustries/AIL11</t>
@@ -867,15 +843,11 @@
           <t>14946</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/leapindialtd/LIL07</t>
@@ -893,7 +865,6 @@
           <t>Technocraft Ventures Ltd</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Closed</t>
@@ -934,15 +905,11 @@
           <t>14840</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/technocraftventuresltd/TVL</t>
@@ -960,7 +927,6 @@
           <t>Dhoot Transmission Ltd</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1001,15 +967,11 @@
           <t>14807</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/dhoottransmissionltd/DTL02</t>
@@ -1027,7 +989,6 @@
           <t>Molbio Diagnostics Ltd</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1068,15 +1029,11 @@
           <t>14526</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/molbiodiagnosticsltd/MDL02</t>
@@ -1094,7 +1051,6 @@
           <t>Milky Mist Dairy Food Ltd</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1135,15 +1091,11 @@
           <t>14980</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/milkymistdairyfoodltd/MMD</t>
@@ -1161,7 +1113,6 @@
           <t>Behari Lal Engineering Ltd</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1202,11 +1153,6 @@
           <t>14820</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/beharilalengineeringltd/BLE</t>
@@ -1224,7 +1170,6 @@
           <t>Shiprocket Ltd</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1265,11 +1210,6 @@
           <t>14938</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/shiprocketltd/SL26</t>
@@ -1287,7 +1227,6 @@
           <t>Lalithaa Jewellery Mart Ltd</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1328,11 +1267,6 @@
           <t>14874</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/lalithaajewellerymartltd/LJML</t>
@@ -1350,7 +1284,6 @@
           <t>Shankesh Jewellers Ltd</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1391,11 +1324,6 @@
           <t>14880</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/shankeshjewellersltd/SJL01</t>
@@ -1413,7 +1341,6 @@
           <t>Sunshine Pictures Ltd</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1454,11 +1381,6 @@
           <t>14760</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/sunshinepicturesltd/SPL13</t>
@@ -1476,7 +1398,6 @@
           <t>Credent Connect N Care Ltd</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1497,7 +1418,6 @@
           <t>Aug 18, 2026</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>600</t>
@@ -1513,11 +1433,6 @@
           <t>113400</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/credentconnectncareltd/CCC04</t>
@@ -1535,7 +1450,6 @@
           <t>Q&amp;T Foods Ltd</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1556,7 +1470,6 @@
           <t>Aug 17, 2026</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>1200</t>
@@ -1572,11 +1485,6 @@
           <t>138000</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/qtfoodsltd/QFL</t>
@@ -1594,7 +1502,6 @@
           <t>Technocrats Plasma Systems Ltd</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Upcoming</t>
@@ -1615,7 +1522,6 @@
           <t>Aug 19, 2026</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>1000</t>
@@ -1631,11 +1537,6 @@
           <t>132000</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>https://www.moneycontrol.com/ipo/technocratsplasmasystemsltd/TPSL</t>

</xml_diff>

<commit_message>
chore: set ipo allotment for Technocraft Ventures Ltd
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -865,6 +865,11 @@
           <t>Technocraft Ventures Ltd</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Closed</t>

</xml_diff>

<commit_message>
feat: update 'got_ipo' status for multiple companies to include 'N/A'
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="82">
   <si>
     <t>company_name</t>
   </si>
@@ -67,42 +67,48 @@
     <t>Juniper Green Energy</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Listed</t>
+  </si>
+  <si>
+    <t>Aug 06, 2026</t>
+  </si>
+  <si>
+    <t>https://www.moneycontrol.com/ipo/renewables/junipergreenenergy/JGE</t>
+  </si>
+  <si>
+    <t>MV Electrosystems</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>https://www.moneycontrol.com/ipo/electric-equipment-switchgears/mvelectrosystems/MEL04</t>
+  </si>
+  <si>
+    <t>Anawil Wire &amp; Engineering</t>
+  </si>
+  <si>
+    <t>Aug 06, 2025</t>
+  </si>
+  <si>
+    <t>Aug 10, 2026</t>
+  </si>
+  <si>
+    <t>https://www.moneycontrol.com/ipo/infrastructure/anawilwireengineering/AWEL</t>
+  </si>
+  <si>
+    <t>2026-08-10 10:24:29</t>
+  </si>
+  <si>
+    <t>Ardee Industries</t>
+  </si>
+  <si>
     <t>No</t>
   </si>
   <si>
-    <t>Listed</t>
-  </si>
-  <si>
-    <t>Aug 06, 2026</t>
-  </si>
-  <si>
-    <t>https://www.moneycontrol.com/ipo/renewables/junipergreenenergy/JGE</t>
-  </si>
-  <si>
-    <t>MV Electrosystems</t>
-  </si>
-  <si>
-    <t>https://www.moneycontrol.com/ipo/electric-equipment-switchgears/mvelectrosystems/MEL04</t>
-  </si>
-  <si>
-    <t>Anawil Wire &amp; Engineering</t>
-  </si>
-  <si>
-    <t>Aug 06, 2025</t>
-  </si>
-  <si>
-    <t>Aug 10, 2026</t>
-  </si>
-  <si>
-    <t>https://www.moneycontrol.com/ipo/infrastructure/anawilwireengineering/AWEL</t>
-  </si>
-  <si>
-    <t>2026-08-10 10:24:29</t>
-  </si>
-  <si>
-    <t>Ardee Industries</t>
-  </si>
-  <si>
     <t>Aug 12, 2026</t>
   </si>
   <si>
@@ -113,9 +119,6 @@
   </si>
   <si>
     <t>LEAP India Ltd</t>
-  </si>
-  <si>
-    <t>Yes</t>
   </si>
   <si>
     <t>Closed</t>
@@ -786,7 +789,7 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>19</v>
@@ -819,12 +822,12 @@
         <v>22</v>
       </c>
       <c r="P3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
@@ -833,10 +836,10 @@
         <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4">
         <v>400</v>
@@ -851,27 +854,27 @@
         <v>139</v>
       </c>
       <c r="P4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Q4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H5">
         <v>281</v>
@@ -886,33 +889,33 @@
         <v>134</v>
       </c>
       <c r="P5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H6">
         <v>94</v>
@@ -927,33 +930,33 @@
         <v>8</v>
       </c>
       <c r="P6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H7">
         <v>70</v>
@@ -968,30 +971,30 @@
         <v>39</v>
       </c>
       <c r="P7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="Q7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H8">
         <v>17</v>
@@ -1006,30 +1009,30 @@
         <v>4</v>
       </c>
       <c r="P8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Q8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H9">
         <v>18</v>
@@ -1044,30 +1047,30 @@
         <v>3</v>
       </c>
       <c r="P9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H10">
         <v>107</v>
@@ -1082,30 +1085,30 @@
         <v>1</v>
       </c>
       <c r="P10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="Q10" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H11">
         <v>52</v>
@@ -1117,30 +1120,30 @@
         <v>14820</v>
       </c>
       <c r="P11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H12">
         <v>154</v>
@@ -1152,164 +1155,164 @@
         <v>14938</v>
       </c>
       <c r="P12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Q12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H13">
         <v>74</v>
       </c>
       <c r="I13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J13">
         <v>14874</v>
       </c>
       <c r="P13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Q13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H14">
         <v>160</v>
       </c>
       <c r="I14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J14">
         <v>14880</v>
       </c>
       <c r="P14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H15">
         <v>41</v>
       </c>
       <c r="I15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J15">
         <v>14760</v>
       </c>
       <c r="P15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q15" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H16">
         <v>600</v>
       </c>
       <c r="I16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J16">
         <v>113400</v>
       </c>
       <c r="P16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H17">
         <v>1200</v>
@@ -1321,42 +1324,42 @@
         <v>138000</v>
       </c>
       <c r="P17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H18">
         <v>1000</v>
       </c>
       <c r="I18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J18">
         <v>132000</v>
       </c>
       <c r="P18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q18" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update IPO data with listing price and gains in JSON file
</commit_message>
<xml_diff>
--- a/data/mainboard_ipos.xlsx
+++ b/data/mainboard_ipos.xlsx
@@ -885,8 +885,20 @@
       <c r="J5">
         <v>14893</v>
       </c>
+      <c r="K5">
+        <v>72</v>
+      </c>
+      <c r="L5">
+        <v>20232</v>
+      </c>
       <c r="M5">
         <v>134</v>
+      </c>
+      <c r="N5">
+        <v>5339</v>
+      </c>
+      <c r="O5">
+        <v>36</v>
       </c>
       <c r="P5" t="s">
         <v>33</v>

</xml_diff>